<commit_message>
Eclipse League: jornada 1 de los grupos A y B (tabla, resultados y numeros por jugador)
</commit_message>
<xml_diff>
--- a/eclipse-numeros.xlsx
+++ b/eclipse-numeros.xlsx
@@ -493,7 +493,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Después de la jornada 1 del Grupo A (lunes 21 de septiembre de 2026). El Grupo B juega el martes 22.</t>
+          <t>Después de la jornada 1: Grupo A el lunes 21 y Grupo B el martes 22 de septiembre de 2026.</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -712,7 +712,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Eclipse League 2026 · Grupo B · Después de la jornada 1 del Grupo A (lunes 21 de septiembre de 2026). El Grupo B juega el martes 22.</t>
+          <t>Eclipse League 2026 · Grupo B · Después de la jornada 1: Grupo A el lunes 21 y Grupo B el martes 22 de septiembre de 2026.</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,666 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Todavía no ha jugado.</t>
+          <t>Jorge Gonzalez</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Oscar Ruyery</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>2</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Janio Tuñon</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>.750</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ricardo Martin</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>.750</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Eliecer Chirino</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>.750</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Francis Guerra</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>.667</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Jose Castillo</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>.500</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Oscar Miranda</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>.500</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Andres Samudio</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>.333</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Daniel Torrealba</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>.333</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Kike Garrido</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>2</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>.333</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Carlos Hernandez</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Isaac Coronado</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Selecta Rookie</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Jair Varela</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>14.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Sotolongo</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>7.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Luis Marin</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
+        <v>1</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Total del equipo</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>.553</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>7.000</t>
         </is>
       </c>
     </row>
@@ -806,7 +1465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -823,7 +1482,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Eclipse League 2026 · Grupo B · Después de la jornada 1 del Grupo A (lunes 21 de septiembre de 2026). El Grupo B juega el martes 22.</t>
+          <t>Eclipse League 2026 · Grupo B · Después de la jornada 1: Grupo A el lunes 21 y Grupo B el martes 22 de septiembre de 2026.</t>
         </is>
       </c>
     </row>
@@ -902,7 +1561,656 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Todavía no ha jugado.</t>
+          <t>Cesar Noguera</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Gigantes</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Luis Alvarez</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Gigantes</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Jose Suira</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Gigantes</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>.667</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Elvis Matute</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Gigantes</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>.500</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Ernesto Corpas</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Gigantes</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>.333</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Fernando Silvera</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Gigantes</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>.333</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Uvaldo Manzane Jr</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Gigantes</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>.333</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Jose Miguel Franco</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Gigantes</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Geovany Cubilla</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Gigantes</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Alexis Otero</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Gigantes</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Cesar Tenorio</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Gigantes</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Felix Herrera</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Gigantes</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Uvaldo Manzane</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Gigantes</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Cesar Tenorio</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Gigantes</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Uvaldo Manzane</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Gigantes</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Luis Alvarez</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Gigantes</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Eduardo Pardo</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Gigantes</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>10.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Total del equipo</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>.370</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>7.000</t>
         </is>
       </c>
     </row>
@@ -917,7 +2225,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -934,7 +2242,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Eclipse League 2026 · Grupo B · Después de la jornada 1 del Grupo A (lunes 21 de septiembre de 2026). El Grupo B juega el martes 22.</t>
+          <t>Eclipse League 2026 · Grupo B · Después de la jornada 1: Grupo A el lunes 21 y Grupo B el martes 22 de septiembre de 2026.</t>
         </is>
       </c>
     </row>
@@ -1013,7 +2321,524 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Todavía no ha jugado.</t>
+          <t>Nicolas Puga</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Pacific Sharks</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Christian Sealy</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Pacific Sharks</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>.667</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>David Quiroz</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Pacific Sharks</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>.667</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Rolando Achurra</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Pacific Sharks</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>.667</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Carlo Real</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Pacific Sharks</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>.333</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Jhon Rojas</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Pacific Sharks</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Fabio Navarro</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Pacific Sharks</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Joshua Quiroz</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Pacific Sharks</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Fidel Ruiz</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Pacific Sharks</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Gunter Chavez</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Pacific Sharks</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Dan Diaz</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Pacific Sharks</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Jhon Galviz</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Pacific Sharks</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>14.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Jorge Brandaris</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Pacific Sharks</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>5.600</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Total del equipo</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>.360</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>7.000</t>
         </is>
       </c>
     </row>
@@ -1028,7 +2853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1045,7 +2870,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Eclipse League 2026 · Grupo B · Después de la jornada 1 del Grupo A (lunes 21 de septiembre de 2026). El Grupo B juega el martes 22.</t>
+          <t>Eclipse League 2026 · Grupo B · Después de la jornada 1: Grupo A el lunes 21 y Grupo B el martes 22 de septiembre de 2026.</t>
         </is>
       </c>
     </row>
@@ -1124,7 +2949,638 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Todavía no ha jugado.</t>
+          <t>Brandon Hernadez</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Pinoleros</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Bryan Florez</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Pinoleros</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Josue Obando</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Pinoleros</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Jose Ortiz</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Pinoleros</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>.667</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Axel Rivas</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Pinoleros</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>.667</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Luis Grijalba</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Pinoleros</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>.500</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Danny Ruiz</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Pinoleros</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>.333</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Jose Brenes</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Pinoleros</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>3</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>.333</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Mario Montoya</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Pinoleros</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Rodrigo Mejia</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Pinoleros</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Edwin Machado</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Pinoleros</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Kevin Obando</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Pinoleros</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Francisco Gutierrez</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Pinoleros</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Leo Hernandez</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Pinoleros</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Luis Grijalba</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Pinoleros</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>7.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Francisco Gutierrez</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Pinoleros</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>4.667</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Total del equipo</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>.393</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>5.833</t>
         </is>
       </c>
     </row>
@@ -1139,7 +3595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1156,7 +3612,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Eclipse League 2026 · Grupo B · Después de la jornada 1 del Grupo A (lunes 21 de septiembre de 2026). El Grupo B juega el martes 22.</t>
+          <t>Eclipse League 2026 · Grupo B · Después de la jornada 1: Grupo A el lunes 21 y Grupo B el martes 22 de septiembre de 2026.</t>
         </is>
       </c>
     </row>
@@ -1235,7 +3691,638 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Todavía no ha jugado.</t>
+          <t>Nino Terriente</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Los Goofis</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Sergio Gonzalez</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Los Goofis</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Randy Saez</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Los Goofis</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Alfredo Padron</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Los Goofis</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sebastian Mirones</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Los Goofis</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Fernando Pitti</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Los Goofis</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>.667</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Luis Silva</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Los Goofis</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>.500</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Dexter Bultron</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Los Goofis</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>.333</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Michael Castellano</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Los Goofis</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>.333</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Alexis Hartman</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Los Goofis</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Francisco Cardenas</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Los Goofis</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Miguel Gonzalez</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Los Goofis</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Luis Mendez</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Los Goofis</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Neomar Perez</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Los Goofis</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Randy Saez</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Los Goofis</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Neomar Perez</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Los Goofis</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>11.31</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Total del equipo</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>.462</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>8.167</t>
         </is>
       </c>
     </row>
@@ -1250,7 +4337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1267,7 +4354,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Eclipse League 2026 · Grupo B · Después de la jornada 1 del Grupo A (lunes 21 de septiembre de 2026). El Grupo B juega el martes 22.</t>
+          <t>Eclipse League 2026 · Grupo B · Después de la jornada 1: Grupo A el lunes 21 y Grupo B el martes 22 de septiembre de 2026.</t>
         </is>
       </c>
     </row>
@@ -1346,7 +4433,686 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Todavía no ha jugado.</t>
+          <t>Alexis Galvez</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Los Panas Soff</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Miguel Caridad</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Los Panas Soff</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>2</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Julio Palacios</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Los Panas Soff</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Jairo Pinto</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Los Panas Soff</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Alvaro Diaz</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Los Panas Soff</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>.500</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Oscar Medina</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Los Panas Soff</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>.333</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Manuel Gamboa</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Los Panas Soff</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Rainer Escorcia</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Los Panas Soff</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Varmore Vega</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Los Panas Soff</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Luis Salazar</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Los Panas Soff</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Victor Lewis</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Los Panas Soff</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Joel Rodriguez</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Los Panas Soff</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Rafael Montilla</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Los Panas Soff</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Richard Escorcia</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Los Panas Soff</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Kendri Maldonado</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Los Panas Soff</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Frederick Pinto</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Los Panas Soff</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Manuel Gamboa</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Los Panas Soff</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>7.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Total del equipo</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>.393</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>7.000</t>
         </is>
       </c>
     </row>
@@ -1826,7 +5592,7 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C15" s="5" t="n">
         <v>0</v>
@@ -1836,7 +5602,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -1845,17 +5611,17 @@
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr">
@@ -1865,18 +5631,18 @@
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>0-0</t>
+          <t>1-0</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Gigantes</t>
+          <t>Pinoleros</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C16" s="5" t="n">
         <v>0</v>
@@ -1886,7 +5652,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -1895,17 +5661,17 @@
         </is>
       </c>
       <c r="G16" s="5" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -1915,7 +5681,7 @@
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>0-0</t>
+          <t>1-0</t>
         </is>
       </c>
     </row>
@@ -1926,7 +5692,7 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C17" s="5" t="n">
         <v>0</v>
@@ -1936,7 +5702,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -1945,17 +5711,17 @@
         </is>
       </c>
       <c r="G17" s="5" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
@@ -1965,52 +5731,52 @@
       </c>
       <c r="L17" s="5" t="inlineStr">
         <is>
-          <t>0-0</t>
+          <t>1-0</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Pinoleros</t>
+          <t>Gigantes</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C18" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D18" s="5" t="n">
         <v>0</v>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>0.000</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G18" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>0-0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="L18" s="5" t="inlineStr">
@@ -2029,38 +5795,38 @@
         <v>0</v>
       </c>
       <c r="C19" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>0.000</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G19" s="5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr">
         <is>
-          <t>0-0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="L19" s="5" t="inlineStr">
@@ -2079,38 +5845,38 @@
         <v>0</v>
       </c>
       <c r="C20" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D20" s="5" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>0.000</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G20" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0</v>
+        <v>-6</v>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>0-0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="L20" s="5" t="inlineStr">
@@ -2130,7 +5896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2310,6 +6076,120 @@
       <c r="H7" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>mar 22 sep</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>7:00 pm</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Pinoleros</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>9</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Los Goofis</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>5</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>mar 22 sep</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>8:20 pm</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Pacific Sharks</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>7</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Gigantes</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>mar 22 sep</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>9:40 pm</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>12</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Los Panas Soff</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>6</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -2341,7 +6221,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Eclipse League 2026 · Grupo A · Después de la jornada 1 del Grupo A (lunes 21 de septiembre de 2026). El Grupo B juega el martes 22.</t>
+          <t>Eclipse League 2026 · Grupo A · Después de la jornada 1: Grupo A el lunes 21 y Grupo B el martes 22 de septiembre de 2026.</t>
         </is>
       </c>
     </row>
@@ -3093,7 +6973,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Eclipse League 2026 · Grupo A · Después de la jornada 1 del Grupo A (lunes 21 de septiembre de 2026). El Grupo B juega el martes 22.</t>
+          <t>Eclipse League 2026 · Grupo A · Después de la jornada 1: Grupo A el lunes 21 y Grupo B el martes 22 de septiembre de 2026.</t>
         </is>
       </c>
     </row>
@@ -3787,7 +7667,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Eclipse League 2026 · Grupo A · Después de la jornada 1 del Grupo A (lunes 21 de septiembre de 2026). El Grupo B juega el martes 22.</t>
+          <t>Eclipse League 2026 · Grupo A · Después de la jornada 1: Grupo A el lunes 21 y Grupo B el martes 22 de septiembre de 2026.</t>
         </is>
       </c>
     </row>
@@ -4615,7 +8495,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Eclipse League 2026 · Grupo A · Después de la jornada 1 del Grupo A (lunes 21 de septiembre de 2026). El Grupo B juega el martes 22.</t>
+          <t>Eclipse League 2026 · Grupo A · Después de la jornada 1: Grupo A el lunes 21 y Grupo B el martes 22 de septiembre de 2026.</t>
         </is>
       </c>
     </row>
@@ -5291,7 +9171,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Eclipse League 2026 · Grupo A · Después de la jornada 1 del Grupo A (lunes 21 de septiembre de 2026). El Grupo B juega el martes 22.</t>
+          <t>Eclipse League 2026 · Grupo A · Después de la jornada 1: Grupo A el lunes 21 y Grupo B el martes 22 de septiembre de 2026.</t>
         </is>
       </c>
     </row>
@@ -5995,7 +9875,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Eclipse League 2026 · Grupo A · Después de la jornada 1 del Grupo A (lunes 21 de septiembre de 2026). El Grupo B juega el martes 22.</t>
+          <t>Eclipse League 2026 · Grupo A · Después de la jornada 1: Grupo A el lunes 21 y Grupo B el martes 22 de septiembre de 2026.</t>
         </is>
       </c>
     </row>

</xml_diff>